<commit_message>
Test ECG EEG and BATT done
</commit_message>
<xml_diff>
--- a/Rerefencia tensiones entrada.xlsx
+++ b/Rerefencia tensiones entrada.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Universidad\STRIKE\MSP430FG479\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895A7579-0B70-4282-A7EF-B3D1B2059575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EDD4186-F5E1-4A37-A80C-B99066FEA8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D4480093-F1CA-4DE4-A6D7-23C3D0A7A5E3}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{D4480093-F1CA-4DE4-A6D7-23C3D0A7A5E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>Vref</t>
   </si>
@@ -69,12 +69,36 @@
   </si>
   <si>
     <t>Vref_real</t>
+  </si>
+  <si>
+    <t>DeltaV</t>
+  </si>
+  <si>
+    <t>EEG1</t>
+  </si>
+  <si>
+    <t>EEG2</t>
+  </si>
+  <si>
+    <t>EEG3</t>
+  </si>
+  <si>
+    <t>ECG</t>
+  </si>
+  <si>
+    <t>BATT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="171" formatCode="0E+00"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -84,12 +108,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -104,8 +146,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,178 +499,293 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F3BD7F-949D-4C48-84C3-F4D6C5FB4091}">
-  <dimension ref="A3:H13"/>
+  <dimension ref="A3:N20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="7" width="24.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5546875" customWidth="1"/>
-    <col min="11" max="11" width="12.77734375" customWidth="1"/>
+    <col min="8" max="8" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5546875" customWidth="1"/>
+    <col min="12" max="12" width="12.77734375" customWidth="1"/>
+    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>1</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>3</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
         <f>1.2</f>
         <v>1.2</v>
       </c>
-      <c r="B4">
-        <f>A4/2</f>
-        <v>0.6</v>
-      </c>
-      <c r="C4">
-        <v>0.4</v>
-      </c>
-      <c r="E4">
-        <v>65535</v>
+      <c r="C4" s="2">
+        <f>B4/2</f>
+        <v>0.6</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.59</v>
       </c>
       <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <f>E4*C4/B4</f>
-        <v>43690</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <f t="shared" ref="A5:A8" si="0">1.2</f>
+        <v>65535</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <f>F4*D4/C4</f>
+        <v>64442.750000000007</v>
+      </c>
+      <c r="M4" t="s">
+        <v>11</v>
+      </c>
+      <c r="N4" s="5">
+        <f>C4/F4</f>
+        <v>9.1554131380178534E-6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <f t="shared" ref="B5:B11" si="0">1.2</f>
         <v>1.2</v>
       </c>
-      <c r="B5">
-        <f t="shared" ref="B5:B8" si="1">A5/2</f>
-        <v>0.6</v>
-      </c>
-      <c r="C5">
-        <v>0.35</v>
-      </c>
-      <c r="E5">
-        <v>65535</v>
+      <c r="C5" s="2">
+        <f t="shared" ref="C5:C11" si="1">B5/2</f>
+        <v>0.6</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.43099999999999999</v>
       </c>
       <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <f t="shared" ref="H5:H8" si="2">E5*C5/B5</f>
-        <v>38228.75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6">
+        <v>65535</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <f>D5*F5/C5</f>
+        <v>47075.974999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
         <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
-      <c r="B6">
+      <c r="C6" s="2">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="C6">
-        <v>0.26</v>
-      </c>
-      <c r="E6">
-        <v>65535</v>
+      <c r="D6" s="3">
+        <v>0.28699999999999998</v>
       </c>
       <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <f t="shared" si="2"/>
-        <v>28398.500000000004</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7">
+        <v>65535</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <f>F6*D6/C6</f>
+        <v>31347.574999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
         <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
-      <c r="B7">
+      <c r="C7" s="2">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="C7">
-        <v>0.2</v>
-      </c>
-      <c r="E7">
-        <v>65535</v>
+      <c r="D7" s="3">
+        <v>0.155</v>
       </c>
       <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <f t="shared" si="2"/>
-        <v>21845</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8">
+        <v>65535</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <f>F7*D7/C7</f>
+        <v>16929.875</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="6">
         <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
-      <c r="B8">
+      <c r="C8" s="7">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="C8">
-        <v>0.2</v>
-      </c>
-      <c r="E8">
-        <v>65535</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="H8">
+      <c r="D8" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6">
+        <v>65535</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="9">
+        <f t="shared" ref="I8:I11" si="2">F8*D8/C8</f>
+        <v>65535</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="10">
+        <f t="shared" si="0"/>
+        <v>1.2</v>
+      </c>
+      <c r="C9" s="11">
+        <f>B9/2</f>
+        <v>0.6</v>
+      </c>
+      <c r="D9" s="12">
+        <v>0.33200000000000002</v>
+      </c>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10">
+        <v>65535</v>
+      </c>
+      <c r="G9" s="10">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10"/>
+      <c r="I9" s="13">
         <f t="shared" si="2"/>
-        <v>21845</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G10" t="s">
+        <v>36262.700000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="14">
+        <f t="shared" si="0"/>
+        <v>1.2</v>
+      </c>
+      <c r="C10" s="15">
+        <f t="shared" si="1"/>
+        <v>0.6</v>
+      </c>
+      <c r="D10" s="16">
+        <v>0.1</v>
+      </c>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14">
+        <v>65535</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="17">
+        <f t="shared" si="2"/>
+        <v>10922.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C11" s="2"/>
+      <c r="D11" s="3"/>
+      <c r="I11" s="1"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
         <v>6</v>
       </c>
-      <c r="H10" t="s">
+      <c r="D15" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="H11">
-        <v>65405</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G12" t="s">
+      <c r="F15" t="s">
         <v>8</v>
       </c>
-      <c r="H12" t="s">
+      <c r="G15" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="H13">
-        <f>H11*B4/E4</f>
-        <v>0.59880979629205766</v>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D16">
+        <v>65535</v>
+      </c>
+      <c r="G16" s="4">
+        <f>D16*C4/F4</f>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="17" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D17">
+        <v>47484</v>
+      </c>
+      <c r="G17" s="4">
+        <f>D17*C5/F5</f>
+        <v>0.4347356374456397</v>
+      </c>
+    </row>
+    <row r="18" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D18">
+        <v>37156</v>
+      </c>
+      <c r="G18" s="4">
+        <f>D18*C6/F6</f>
+        <v>0.34017853055619135</v>
+      </c>
+    </row>
+    <row r="19" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D19">
+        <v>21856</v>
+      </c>
+      <c r="G19" s="4">
+        <f>D19*C7/F7</f>
+        <v>0.2001007095445182</v>
+      </c>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="G20" s="4">
+        <f>D20*C8/F8</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>